<commit_message>
feat: add 관리구분 header column to bulk templates
</commit_message>
<xml_diff>
--- a/development/service-ops-api/src/main/resources/templates/excel/matching-template.xlsx
+++ b/development/service-ops-api/src/main/resources/templates/excel/matching-template.xlsx
@@ -9,9 +9,16 @@
   <sheets>
     <sheet name="차량-라이더 매칭" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="1">
+  <si>
+    <t>관리구분 (삭제 시 '삭제' 입력)</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -564,18 +571,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I500"/>
+  <dimension ref="A1:J500"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
+    <col min="1" max="1" customWidth="true" width="16.0"/>
+    <col min="2" max="2" customWidth="true" width="16.0"/>
+    <col min="3" max="3" customWidth="true" width="16.0"/>
+    <col min="4" max="4" customWidth="true" width="18.0"/>
+    <col min="5" max="5" customWidth="true" width="14.0"/>
+    <col min="6" max="6" customWidth="true" width="16.0"/>
+    <col min="7" max="7" customWidth="true" width="16.0"/>
+    <col min="8" max="8" customWidth="true" width="16.0"/>
+    <col min="9" max="9" customWidth="true" width="20.0"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -584,6 +591,7 @@
           <t>※ 이 파일은 시스템에서 현재 등록된 차량·라이더 목록을 기반으로 자동 생성됩니다. 차량번호와 라이더이름은 드롭다운에서 선택하세요. ⚠️ 표시 행은 문제가 있는 매칭입니다 — 수정 후 저장하거나 삭제하세요.</t>
         </is>
       </c>
+      <c r="J1" s="0"/>
     </row>
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -657,6 +665,9 @@
           <t>검증 결과</t>
         </is>
       </c>
+      <c r="J3" t="s" s="0">
+        <v>0</v>
+      </c>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="10" t="inlineStr">

</xml_diff>

<commit_message>
Revert "Merge pull request #484 from EVNSolution/cc-107-excel-bulk-delete"
This reverts commit fba9df814e81ceb065790289e745faea9a2a1e34, reversing
changes made to 12288c1065c30b60a6762a0812a27863a2205620.
</commit_message>
<xml_diff>
--- a/development/service-ops-api/src/main/resources/templates/excel/matching-template.xlsx
+++ b/development/service-ops-api/src/main/resources/templates/excel/matching-template.xlsx
@@ -9,16 +9,9 @@
   <sheets>
     <sheet name="차량-라이더 매칭" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
-</file>
-
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="1">
-  <si>
-    <t>관리구분 (삭제 시 '삭제' 입력)</t>
-  </si>
-</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -571,18 +564,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J500"/>
+  <dimension ref="A1:I500"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="16.0"/>
-    <col min="2" max="2" customWidth="true" width="16.0"/>
-    <col min="3" max="3" customWidth="true" width="16.0"/>
-    <col min="4" max="4" customWidth="true" width="18.0"/>
-    <col min="5" max="5" customWidth="true" width="14.0"/>
-    <col min="6" max="6" customWidth="true" width="16.0"/>
-    <col min="7" max="7" customWidth="true" width="16.0"/>
-    <col min="8" max="8" customWidth="true" width="16.0"/>
-    <col min="9" max="9" customWidth="true" width="20.0"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -591,7 +584,6 @@
           <t>※ 이 파일은 시스템에서 현재 등록된 차량·라이더 목록을 기반으로 자동 생성됩니다. 차량번호와 라이더이름은 드롭다운에서 선택하세요. ⚠️ 표시 행은 문제가 있는 매칭입니다 — 수정 후 저장하거나 삭제하세요.</t>
         </is>
       </c>
-      <c r="J1" s="0"/>
     </row>
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -665,9 +657,6 @@
           <t>검증 결과</t>
         </is>
       </c>
-      <c r="J3" t="s" s="0">
-        <v>0</v>
-      </c>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="10" t="inlineStr">

</xml_diff>